<commit_message>
modernize staging CI runtime
</commit_message>
<xml_diff>
--- a/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
+++ b/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nevada-my.sharepoint.com/personal/pshill_unr_edu/Documents/Robotics-Programming-Lab-v4/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nevada-my.sharepoint.com/personal/pshill_unr_edu/Documents/Robotics-Programming-Lab-Staging/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2749" documentId="13_ncr:1_{18EF0F70-DCE6-4CF6-A4C9-67DAEC6D01BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0230118-C4B2-41B8-992A-5884BF312F28}"/>
+  <xr:revisionPtr revIDLastSave="2753" documentId="13_ncr:1_{18EF0F70-DCE6-4CF6-A4C9-67DAEC6D01BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A85715D9-3685-4CDD-B51C-C6CA2CFFE131}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21840" xr2:uid="{BB5C9DB2-203A-4056-840F-F797153FBD4E}"/>
   </bookViews>
@@ -4571,12 +4571,6 @@
     <t>GitHub Actions</t>
   </si>
   <si>
-    <t>CI now includes repository safety, PostgreSQL migration, backend, Flutter, and sandbox Docker image smoke jobs.</t>
-  </si>
-  <si>
-    <t>Run and verify after the initial staging main push.</t>
-  </si>
-  <si>
     <t>Staging</t>
   </si>
   <si>
@@ -4656,6 +4650,12 @@
   </si>
   <si>
     <t>Initial staging candidate; SHA recorded in Git/GitHub</t>
+  </si>
+  <si>
+    <t>Hosted run 30895379726 passed repository safety, backend/PostgreSQL migration, Flutter, and sandbox image build/smoke jobs.</t>
+  </si>
+  <si>
+    <t>Node 20 maintenance warnings were addressed with official actions v7; final commit rerun required.</t>
   </si>
 </sst>
 </file>
@@ -8178,10 +8178,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{507B0FA5-A9A9-47C1-A4F2-AA863A2D1168}" name="V4SqaResults" displayName="V4SqaResults" ref="A12:F58" totalsRowShown="0" headerRowDxfId="181" dataDxfId="180">
   <autoFilter ref="A12:F58" xr:uid="{507B0FA5-A9A9-47C1-A4F2-AA863A2D1168}"/>
@@ -8680,7 +8676,7 @@
         <v>924</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>1531</v>
+        <v>1529</v>
       </c>
       <c r="C4" s="33" t="s">
         <v>1254</v>
@@ -8728,14 +8724,14 @@
       </c>
       <c r="D7" s="38">
         <f>COUNTIF(C13:C58,"Pass")</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" s="36" t="s">
         <v>1256</v>
       </c>
       <c r="F7" s="36">
         <f>B7-D7</f>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -8744,7 +8740,7 @@
       </c>
       <c r="B8" s="37">
         <f>IF(B7=0,0,D7/B7)</f>
-        <v>0.78260869565217395</v>
+        <v>0.80434782608695654</v>
       </c>
       <c r="C8" s="36" t="s">
         <v>36</v>
@@ -8758,7 +8754,7 @@
       </c>
       <c r="F8" s="38">
         <f>COUNTIF(C13:C58,"Not Run")+COUNTIF(C13:C58,"Deferred")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -9702,16 +9698,16 @@
         <v>1501</v>
       </c>
       <c r="C58" s="31" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D58" s="31" t="s">
         <v>1502</v>
       </c>
       <c r="E58" s="31" t="s">
-        <v>1503</v>
+        <v>1530</v>
       </c>
       <c r="F58" s="31" t="s">
-        <v>1504</v>
+        <v>1531</v>
       </c>
     </row>
   </sheetData>
@@ -41410,100 +41406,100 @@
     </row>
     <row r="37" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>1505</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="D37" s="19" t="s">
         <v>1506</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>1507</v>
-      </c>
-      <c r="D37" s="19" t="s">
-        <v>1508</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
-        <v>1505</v>
+        <v>1503</v>
       </c>
       <c r="B38" s="9" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>1508</v>
+      </c>
+      <c r="D38" s="19" t="s">
         <v>1509</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>1510</v>
-      </c>
-      <c r="D38" s="19" t="s">
-        <v>1511</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">
-        <v>1505</v>
+        <v>1503</v>
       </c>
       <c r="B39" s="9" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>1511</v>
+      </c>
+      <c r="D39" s="19" t="s">
         <v>1512</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>1513</v>
-      </c>
-      <c r="D39" s="19" t="s">
-        <v>1514</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="21" t="s">
+        <v>1513</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>1514</v>
+      </c>
+      <c r="C40" s="9" t="s">
         <v>1515</v>
       </c>
-      <c r="B40" s="9" t="s">
+      <c r="D40" s="19" t="s">
         <v>1516</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>1517</v>
-      </c>
-      <c r="D40" s="19" t="s">
-        <v>1518</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
+        <v>1517</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C41" s="9" t="s">
         <v>1519</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="D41" s="19" t="s">
         <v>1520</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>1521</v>
-      </c>
-      <c r="D41" s="19" t="s">
-        <v>1522</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
+        <v>1521</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>1522</v>
+      </c>
+      <c r="C42" s="9" t="s">
         <v>1523</v>
       </c>
-      <c r="B42" s="9" t="s">
+      <c r="D42" s="19" t="s">
         <v>1524</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>1525</v>
-      </c>
-      <c r="D42" s="19" t="s">
-        <v>1526</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="21" t="s">
+        <v>1525</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>1526</v>
+      </c>
+      <c r="C43" s="9" t="s">
         <v>1527</v>
       </c>
-      <c r="B43" s="9" t="s">
+      <c r="D43" s="19" t="s">
         <v>1528</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>1529</v>
-      </c>
-      <c r="D43" s="19" t="s">
-        <v>1530</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
finalize staging SQA evidence
</commit_message>
<xml_diff>
--- a/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
+++ b/Robotics_Programming_Lab_Master_SQA_Checklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nevada-my.sharepoint.com/personal/pshill_unr_edu/Documents/Robotics-Programming-Lab-Staging/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cspon\OneDrive - University of Nevada, Reno\Robotics-Programming-Lab-Staging\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2753" documentId="13_ncr:1_{18EF0F70-DCE6-4CF6-A4C9-67DAEC6D01BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A85715D9-3685-4CDD-B51C-C6CA2CFFE131}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78FD89A-171B-408E-9D18-D58E47DF8247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21840" xr2:uid="{BB5C9DB2-203A-4056-840F-F797153FBD4E}"/>
   </bookViews>
@@ -4652,10 +4652,10 @@
     <t>Initial staging candidate; SHA recorded in Git/GitHub</t>
   </si>
   <si>
-    <t>Hosted run 30895379726 passed repository safety, backend/PostgreSQL migration, Flutter, and sandbox image build/smoke jobs.</t>
-  </si>
-  <si>
-    <t>Node 20 maintenance warnings were addressed with official actions v7; final commit rerun required.</t>
+    <t>Hosted staging CI passed repository safety, backend/PostgreSQL migration, Flutter, and sandbox image build/smoke jobs.</t>
+  </si>
+  <si>
+    <t>The current staging main SHA must retain a successful hosted run before production promotion.</t>
   </si>
 </sst>
 </file>

</xml_diff>